<commit_message>
feat: tich hop Che do Kiem tra tinh diem, cham diem thang 10 va Bang diem Giao vien vao Website on tap Tin hoc GK1
</commit_message>
<xml_diff>
--- a/Check_các_cuộc_thi/IOE/Lần 1/Thống kê IOE - Lần 1.xlsx
+++ b/Check_các_cuộc_thi/IOE/Lần 1/Thống kê IOE - Lần 1.xlsx
@@ -3601,7 +3601,7 @@
       </c>
       <c r="B126" s="7" t="inlineStr">
         <is>
-          <t>13/09/2013</t>
+          <t>Trần Hải Phong</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>18/10/2014</t>
+          <t>Lê Ngọc Hân</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -3649,7 +3649,7 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>2014-05-02 00:00:00</t>
+          <t>Đỗ Nguyễn Hà Minh</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>2014-04-09 00:00:00</t>
+          <t>Nguyễn Hoàng Hương Trà</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>26/6/2014</t>
+          <t>Bùi Mai Phương</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>2014-09-09 00:00:00</t>
+          <t>Đỗ Trọng Hoàng</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>16/10/2014</t>
+          <t>Trần Đức Tài</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B134" s="7" t="inlineStr">
         <is>
-          <t>30/03/2013</t>
+          <t>Đỗ Tuệ Linh</t>
         </is>
       </c>
       <c r="C134" s="6" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>2013-02-02 00:00:00</t>
+          <t>Nguyễn Quang Hải Nam</t>
         </is>
       </c>
       <c r="C135" s="6" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>2013-02-08 00:00:00</t>
+          <t>Phan Đức Việt</t>
         </is>
       </c>
       <c r="C136" s="6" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="B137" s="7" t="inlineStr">
         <is>
-          <t>2013-08-05 00:00:00</t>
+          <t>Nguyễn Quỳnh Chi</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
-          <t>14/08/2013</t>
+          <t>Trần An Như</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>24/10/2013</t>
+          <t>Nguyễn Minh Thư</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -3927,7 +3927,7 @@
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>2013-05-09 00:00:00</t>
+          <t>Nguyễn Trần Khánh Dương</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>23/9/2013</t>
+          <t>Trần Lê Khánh An</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>2013-04-06 00:00:00</t>
+          <t>Lê Bảo Minh</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t>28/02/2013</t>
+          <t>Nguyễn Nam Phong</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>13/09/2013</t>
+          <t>Trần Hải Phong</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -6996,7 +6996,7 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>18/10/2014</t>
+          <t>Lê Ngọc Hân</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>2014-05-02 00:00:00</t>
+          <t>Đỗ Nguyễn Hà Minh</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>2014-04-09 00:00:00</t>
+          <t>Nguyễn Hoàng Hương Trà</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>26/6/2014</t>
+          <t>Bùi Mai Phương</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>2014-09-09 00:00:00</t>
+          <t>Đỗ Trọng Hoàng</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="B133" s="7" t="inlineStr">
         <is>
-          <t>16/10/2014</t>
+          <t>Trần Đức Tài</t>
         </is>
       </c>
       <c r="C133" s="6" t="inlineStr">
@@ -7161,7 +7161,7 @@
       </c>
       <c r="B137" s="7" t="inlineStr">
         <is>
-          <t>30/03/2013</t>
+          <t>Đỗ Tuệ Linh</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
@@ -7182,7 +7182,7 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
-          <t>2013-02-02 00:00:00</t>
+          <t>Nguyễn Quang Hải Nam</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>2013-02-08 00:00:00</t>
+          <t>Phan Đức Việt</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>2013-08-05 00:00:00</t>
+          <t>Nguyễn Quỳnh Chi</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>14/08/2013</t>
+          <t>Trần An Như</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>24/10/2013</t>
+          <t>Nguyễn Minh Thư</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t>2013-05-09 00:00:00</t>
+          <t>Nguyễn Trần Khánh Dương</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="B144" s="7" t="inlineStr">
         <is>
-          <t>23/9/2013</t>
+          <t>Trần Lê Khánh An</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="B145" s="7" t="inlineStr">
         <is>
-          <t>2013-04-06 00:00:00</t>
+          <t>Lê Bảo Minh</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B146" s="7" t="inlineStr">
         <is>
-          <t>28/02/2013</t>
+          <t>Nguyễn Nam Phong</t>
         </is>
       </c>
       <c r="C146" s="6" t="inlineStr">

</xml_diff>